<commit_message>
Release 0.4.1: input validation, strict settings, pandas 3 support, monotone fixes
</commit_message>
<xml_diff>
--- a/examples/outputs/mosaic_export.xlsx
+++ b/examples/outputs/mosaic_export.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,97 +421,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Entity Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>UUID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Reserve Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Product Type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Use Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Segment #</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Start Date T0  (y-m-d)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Initial Rate qi (rate/d)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Final Rate qf (rate/d)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>D Cum</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Final Cum</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Length DT (years)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Final Date Tf  (y-m-d)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Exponent N, b</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Nominal Decline Di (%)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Tangential Effective Decline   Dei (%)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Secant Effective Decline Desi (%)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Service Factor (fraction)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Minimum Effective Decline Dmin (%)</t>
         </is>
@@ -554,11 +542,11 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H2" t="n">
-        <v>3.001434246397276</v>
+        <v>2.910791807102476</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -573,7 +561,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>29.0747202138165</v>
+        <v>27.04935127581817</v>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">
@@ -605,11 +593,11 @@
       <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H3" t="n">
-        <v>7.644433927408456</v>
+        <v>7.334815299450403</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -624,7 +612,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>34.03956555932896</v>
+        <v>32.90767009560411</v>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
@@ -656,11 +644,11 @@
       <c r="F4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H4" t="n">
-        <v>6.072737695865979</v>
+        <v>5.936473200685517</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -670,12 +658,12 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>0.9900000000000001</v>
+        <v>0.9900000000001198</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>21.52396529120245</v>
+        <v>20.17853372987656</v>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
@@ -707,11 +695,11 @@
       <c r="F5" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H5" t="n">
-        <v>4.396554238704987</v>
+        <v>4.283126487056699</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -726,7 +714,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>25.50054100727116</v>
+        <v>24.01566797885962</v>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
@@ -758,11 +746,11 @@
       <c r="F6" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H6" t="n">
-        <v>17.58506932375363</v>
+        <v>17.13116934501094</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -777,7 +765,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>25.49949322069542</v>
+        <v>24.01425683958599</v>
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
@@ -809,11 +797,11 @@
       <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H7" t="n">
-        <v>7.708567187724205</v>
+        <v>7.573055532607241</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -828,7 +816,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>19.07570122045679</v>
+        <v>17.77735608620902</v>
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
@@ -860,11 +848,11 @@
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H8" t="n">
-        <v>2.271847902691497</v>
+        <v>2.189122280835324</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -879,7 +867,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>31.70912951565447</v>
+        <v>30.14466555904177</v>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
@@ -911,11 +899,11 @@
       <c r="F9" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H9" t="n">
-        <v>4.637976896035546</v>
+        <v>4.40197521658817</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -930,7 +918,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>38.15954203603814</v>
+        <v>38.16035232824231</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
@@ -962,11 +950,11 @@
       <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="H10" t="n">
-        <v>4.525421084039723</v>
+        <v>4.398802337696591</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -981,7 +969,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>26.04846664655377</v>
+        <v>24.50104328313862</v>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">

</xml_diff>

<commit_message>
Assorted bug fixes and performance improvements.
</commit_message>
<xml_diff>
--- a/examples/outputs/mosaic_export.xlsx
+++ b/examples/outputs/mosaic_export.xlsx
@@ -546,7 +546,7 @@
         <v>44256</v>
       </c>
       <c r="H2" t="n">
-        <v>2.910791807102476</v>
+        <v>2.910823237287937</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -561,7 +561,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>27.04935127581817</v>
+        <v>27.04464337566458</v>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">
@@ -801,7 +801,7 @@
         <v>44256</v>
       </c>
       <c r="H7" t="n">
-        <v>7.573055532607241</v>
+        <v>7.573066094541761</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -816,7 +816,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>17.77735608620902</v>
+        <v>17.77637300440403</v>
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">

</xml_diff>